<commit_message>
Fixed Chunking Mechanism and cleaner logging
</commit_message>
<xml_diff>
--- a/data/Retrieval Insights.xlsx
+++ b/data/Retrieval Insights.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="24">
   <si>
     <t>Parameters</t>
   </si>
@@ -62,7 +62,16 @@
 3. The Principle of Excluded Middle</t>
   </si>
   <si>
+    <t>Highest score one was completely irrelevant.</t>
+  </si>
+  <si>
     <t>rank 6</t>
+  </si>
+  <si>
+    <t>no all above 0.7</t>
+  </si>
+  <si>
+    <t>In the top 6 chunks only last 2 chunks were from the correct source file</t>
   </si>
   <si>
     <t>What does this text say about the impact of Neural Networks on logical inference?</t>
@@ -87,6 +96,9 @@
   </si>
   <si>
     <t>The Law of Simplicity states that combining a logical term with itself does not change its meaning, so repeating the same term has no effect and the result remains the same as the original term.</t>
+  </si>
+  <si>
+    <t>all chunks scored above 0.7, nothing matches except the word logical or inference</t>
   </si>
 </sst>
 </file>
@@ -622,8 +634,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="8" width="22.25"/>
-    <col customWidth="1" min="9" max="28" width="25.75"/>
+    <col customWidth="1" min="1" max="28" width="19.5"/>
   </cols>
   <sheetData>
     <row r="1" ht="84.75" customHeight="1">
@@ -682,12 +693,18 @@
       <c r="C2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
+      <c r="E2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>14</v>
+      </c>
       <c r="H2" s="6"/>
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
@@ -713,10 +730,10 @@
     <row r="3" ht="51.0" customHeight="1">
       <c r="A3" s="4"/>
       <c r="B3" s="4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -747,10 +764,10 @@
     <row r="4" ht="51.0" customHeight="1">
       <c r="A4" s="6"/>
       <c r="B4" s="9" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -781,10 +798,10 @@
     <row r="5" ht="51.0" customHeight="1">
       <c r="A5" s="6"/>
       <c r="B5" s="10" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
@@ -815,10 +832,10 @@
     <row r="6" ht="51.0" customHeight="1">
       <c r="A6" s="6"/>
       <c r="B6" s="9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
@@ -30318,12 +30335,18 @@
       <c r="C2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="6"/>
-      <c r="E2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
+      <c r="E2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>14</v>
+      </c>
       <c r="H2" s="6"/>
       <c r="I2" s="15"/>
       <c r="J2" s="15"/>
@@ -30347,16 +30370,18 @@
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="4"/>
       <c r="B3" s="16" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
+      <c r="H3" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="I3" s="15"/>
       <c r="J3" s="15"/>
       <c r="K3" s="15"/>
@@ -30379,10 +30404,10 @@
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="4"/>
       <c r="B4" s="9" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -30411,10 +30436,10 @@
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="4"/>
       <c r="B5" s="10" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
@@ -30443,10 +30468,10 @@
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="4"/>
       <c r="B6" s="9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>

</xml_diff>